<commit_message>
Update metadata table build: - pull id/names from CEPALSTAT - drop last year and last updated info - generate yearbook flag based on anuario index - define management system in code by data source or id - define notes in code - write to xlsx
</commit_message>
<xml_diff>
--- a/Data/indicator_metadata.xlsx
+++ b/Data/indicator_metadata.xlsx
@@ -15,9 +15,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -55,12 +52,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -355,11 +351,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:K84"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="11" max="11" width="20.7109375" style="2" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
@@ -384,40 +377,35 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>cat3</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>source</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>dimensions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>anuario</t>
-        </is>
-      </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>yearbook</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>profile</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>automated</t>
-        </is>
-      </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>last_run</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -434,24 +422,24 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Physical conditions</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Atmosphere, climate and weather</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>FAO</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Y</t>
@@ -466,88 +454,82 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K2" s="2">
-        <v>45960</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>2035</v>
+        <v>4501</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Country area</t>
+          <t>Lakes and rivers permanent water area (square kilometres) EN_LKRV_PWAN</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Physical conditions</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Geological and geographical characteristics</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>FAO</t>
+          <t>Hydrographical characteristics</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Type of area</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>SDG</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="K3" s="2">
-        <v>45959</v>
+          <t>sdg</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>2054</v>
+        <v>2035</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Area of inland waters</t>
+          <t>Country area</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Physical conditions</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Geological and geographical characteristics</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>Geological and geographical information</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>FAO</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Type of area</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>Y</t>
@@ -557,324 +539,315 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K4" s="2">
-        <v>45999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>4176</v>
+        <v>2054</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mangroves</t>
+          <t>Area of inland waters</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Land cover, ecosystems and biodiversity</t>
+          <t>Environmental conditions and quality</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Land cover</t>
+          <t>Physical conditions</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>Geological and geographical information</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>FAO</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K5" s="2">
-        <v>45968</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>3355</v>
+        <v>3974</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Permanent snow and glaciers</t>
+          <t>Proportion of land that is degraded over total land area (%) AG_LND_DGRD</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Land cover, ecosystems and biodiversity</t>
+          <t>Environmental conditions and quality</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Land cover</t>
+          <t>Physical conditions</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>FAO</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>Soil characteristics</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SDG</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="K6" s="2">
-        <v>45964</v>
+          <t>sdg</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>5417</v>
+        <v>4176</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Land cover ratio</t>
+          <t>Mangrove area</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Land cover</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>ECLAC</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>N</t>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>FAO</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>geo</t>
+          <t>env</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <v>5418</v>
+        <v>2016</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Indice de heterogeneidad de paisaje</t>
+          <t>Area of wetlands designated under the Ramsar Convention</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Land cover</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>ECLAC</t>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Ramsar</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>geo</t>
+          <t>env</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>3963</v>
+        <v>3355</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Average proportion of Marine Key Biodiversity Areas (KBAs) covered by protected areas (%) ER_MRN_MPA</t>
+          <t>Area of permanent snow and glaciers</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Land cover</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>SDG</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>N</t>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>FAO</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>sdg</t>
+          <t>env</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <v>3967</v>
+        <v>5417</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Average proportion of Terrestrial Key Biodiversity Areas (KBAs) covered by protected areas (%) ER_PTD_TERR</t>
+          <t>Area under each land cover class as a proportion of total land area (subnational)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Land cover</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>SDG</t>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ECLAC</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>N</t>
+          <t>Land coverage; Minor administrative division</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>sdg</t>
+          <t>geo</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <v>3968</v>
+        <v>5418</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Average proportion of Freshwater Key Biodiversity Areas (KBAs) covered by protected areas (%) ER_PTD_FRHWTR</t>
+          <t>Landscape heterogeneity index (subnational)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Land cover</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>SDG</t>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>ECLAC</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>N</t>
+          <t>Minor administrative division</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>sdg</t>
+          <t>geo</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>3974</v>
+        <v>3963</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Proportion of land that is degraded over total land area (%) AG_LND_DGRD</t>
+          <t>Average proportion of Marine Key Biodiversity Areas (KBAs) covered by protected areas (%) ER_MRN_MPA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
           <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Land cover</t>
-        </is>
-      </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>Biodiversity</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>SDG</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>N</t>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -885,31 +858,31 @@
     </row>
     <row r="13">
       <c r="A13">
-        <v>2016</v>
+        <v>3967</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Surface area of Ramsar designated wetlands</t>
+          <t>Average proportion of Terrestrial Key Biodiversity Areas (KBAs) covered by protected areas (%) ER_PTD_TERR</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
           <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Ecosystems</t>
-        </is>
-      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ramsar</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>Biodiversity</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>SDG</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -924,45 +897,47 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="K13" s="2">
-        <v>46156</v>
+          <t>sdg</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>3979</v>
+        <v>3968</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Red List Index ER_RSK_LST</t>
+          <t>Average proportion of Freshwater Key Biodiversity Areas (KBAs) covered by protected areas (%) ER_PTD_FRHWTR</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
           <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Biodiversity</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>SDG</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -973,131 +948,125 @@
     </row>
     <row r="15">
       <c r="A15">
-        <v>2036</v>
+        <v>3979</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Forest area, by type of forest</t>
+          <t>Red List Index ER_RSK_LST</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Forest</t>
-        </is>
-      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FAO</t>
+          <t>Biodiversity</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Type of forest</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
+          <t>SDG</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="K15" s="2">
-        <v>45999</v>
+          <t>sdg</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <v>2021</v>
+        <v>2036</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Forest area as a proportion of total land area, by type of forest</t>
+          <t>Forest area, by type of forest</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
           <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Forest</t>
-        </is>
-      </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>Forests</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>FAO</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Type of forest</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K16" s="2">
-        <v>46000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17">
-        <v>2530</v>
+        <v>2021</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Natural forest area as a proportion of total forest</t>
+          <t>Forest area as a proportion of total land area, by type of forest</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Forest</t>
-        </is>
-      </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>FAO</t>
+          <t>Forests</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>ECLAC</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
+          <t>Type of forest</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -1110,41 +1079,38 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K17" s="2">
-        <v>45999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18">
-        <v>2531</v>
+        <v>2530</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Forest plantation area as a proportion of total forest</t>
+          <t>Natural forest area as a proportion of total forest area</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
           <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Forest</t>
-        </is>
-      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FAO</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
+          <t>Forests</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>ECLAC</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1153,43 +1119,45 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K18" s="2">
-        <v>45999</v>
       </c>
     </row>
     <row r="19">
       <c r="A19">
-        <v>5422</v>
+        <v>2531</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Average forest height</t>
+          <t>Forest plantation area as a proportion of total forest area</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Forest</t>
-        </is>
-      </c>
       <c r="E19" t="inlineStr">
         <is>
+          <t>Forests</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>ECLAC</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>N</t>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>geo</t>
+          <t>env</t>
         </is>
       </c>
     </row>
@@ -1199,27 +1167,32 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Forest expanse</t>
+          <t>Forest extent (subnational)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
           <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Forest</t>
-        </is>
-      </c>
       <c r="E20" t="inlineStr">
         <is>
+          <t>Forests</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
           <t>ECLAC</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>N</t>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Minor administrative division</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1234,27 +1207,33 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Extent of Forest Loss</t>
+          <t xml:space="preserve">Extent of forest loss (subnational)
+</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
           <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Forest</t>
-        </is>
-      </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>Forests</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t>ECLAC</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>N</t>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Minor administrative division</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1269,27 +1248,32 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Forest gain extension</t>
+          <t>Extent of forest gain (subnational)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
+          <t>Environmental conditions and quality</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
           <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Forest</t>
-        </is>
-      </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t>Forests</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>ECLAC</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>N</t>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Minor administrative division</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1300,71 +1284,76 @@
     </row>
     <row r="23">
       <c r="A23">
-        <v>3946</v>
+        <v>5422</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Annual mean levels of fine particulate matter (population-weighted), by location (micrograms per cubic meter) EN_ATM_PM25</t>
+          <t>Average forest height (subnational)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Environmental quality</t>
+          <t>Environmental conditions and quality</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Air quality</t>
+          <t>Land cover, ecosystems and biodiversity</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SDG</t>
+          <t>Forests</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>N</t>
+          <t>ECLAC</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Minor administrative division</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>sdg</t>
+          <t>geo</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24">
-        <v>4243</v>
+        <v>3946</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>GDP energy intensity by economic activity</t>
+          <t>Annual mean levels of fine particulate matter (population-weighted), by location (micrograms per cubic meter) EN_ATM_PM25</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Energy resources</t>
+          <t>Environmental conditions and quality</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
+          <t>Environmental quality</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>OLADE</t>
+          <t>Air quality</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Energy intensity_Economic activity</t>
+          <t>SDG</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Location</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1372,115 +1361,79 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="K24" s="2">
-        <v>46142</v>
+          <t>sdg</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25">
-        <v>4150</v>
+        <v>3850</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Installed capacity for producing electricity, by energy source</t>
+          <t>Proportion of bodies of water with good ambient water quality (%) EN_H2O_WBAMBQ</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Energy resources</t>
+          <t>Environmental conditions and quality</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
+          <t>Environmental quality</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>OLADE</t>
+          <t>Fresh water quality</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Type of energy source</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>SDG</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="K25" s="2">
-        <v>46147</v>
+          <t>sdg</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26">
-        <v>4236</v>
+        <v>5672</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Proportion of renewable primary energy supply, by type of energy</t>
+          <t>Energy production</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E26" t="inlineStr">
         <is>
+          <t>Production, trade and consumption of energy</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
           <t>OLADE</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Renewable and non-renewable primary energy type</t>
-        </is>
-      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>Type of energy__Primary_and_Secondary</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1488,37 +1441,44 @@
           <t>env</t>
         </is>
       </c>
-      <c r="K26" s="2">
-        <v>46133</v>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>this used to be indicator 2040</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27">
-        <v>4174</v>
+        <v>2487</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>GDP energy intensity (Primary energy supply / GDP)</t>
+          <t>Primary and secondary energy supply</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E27" t="inlineStr">
         <is>
+          <t>Production, trade and consumption of energy</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
           <t>OLADE</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>Type of energy__Primary_and_Secondary</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1535,9 +1495,6 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K27" s="2">
-        <v>46135</v>
       </c>
     </row>
     <row r="28">
@@ -1546,53 +1503,40 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Energy consumption</t>
+          <t>Final energy consumption</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E28" t="inlineStr">
         <is>
+          <t>Production, trade and consumption of energy</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
           <t>OLADE</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>Type of energy__Primary_and_Secondary</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
           <t>env</t>
         </is>
       </c>
-      <c r="K28" s="2">
-        <v>46135</v>
-      </c>
-      <c r="L28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>this used to be indicator 2041</t>
         </is>
@@ -1600,125 +1544,124 @@
     </row>
     <row r="29">
       <c r="A29">
-        <v>4183</v>
+        <v>2486</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Variation rate of GDP energy intensity (Primary energy supply / GDP)</t>
+          <t>Primary energy supply from renewable and non-renewable sources, by type of energy</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E29" t="inlineStr">
         <is>
+          <t>Renewable energy</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
           <t>OLADE</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Renewable and non-renewable primary energy type</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K29" s="2">
-        <v>46136</v>
       </c>
     </row>
     <row r="30">
       <c r="A30">
-        <v>4244</v>
+        <v>3154</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Public investments trends in renewable energy</t>
+          <t>Renewable energy share of primary energy supply</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E30" t="inlineStr">
         <is>
+          <t>Renewable energy</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
           <t>OLADE</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Type of renewable energy</t>
-        </is>
-      </c>
       <c r="H30" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K30" s="2">
-        <v>46043</v>
       </c>
     </row>
     <row r="31">
       <c r="A31">
-        <v>2486</v>
+        <v>4236</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Primary energy supply from renewable and non-renewable sources, by type of energy</t>
+          <t>Composition of renewable primary energy supply, by type of energy</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E31" t="inlineStr">
         <is>
+          <t>Renewable energy</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
           <t>OLADE</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>Renewable and non-renewable primary energy type</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1732,33 +1675,35 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K31" s="2">
-        <v>46133</v>
       </c>
     </row>
     <row r="32">
       <c r="A32">
-        <v>4184</v>
+        <v>3883</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Variation rate of GDP energy intensity (Final energy consumption / GDP)</t>
+          <t>Renewable energy share in the total final energy consumption (%) EG_FEC_RNEW</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>OLADE</t>
+          <t>Renewable energy</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>SDG</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1773,35 +1718,37 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="K32" s="2">
-        <v>46139</v>
+          <t>sdg</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33">
-        <v>4234</v>
+        <v>4174</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Electricity losses</t>
+          <t>Energy intensity measured in terms of primary energy and GDP</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>OLADE</t>
+          <t>Energy efficiency</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>ECLAC</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1818,45 +1765,37 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K33" s="2">
-        <v>46146</v>
       </c>
     </row>
     <row r="34">
       <c r="A34">
-        <v>4235</v>
+        <v>4183</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Proportion of electricity losses</t>
+          <t>Change in energy intensity measured in terms of primary energy and GDP</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E34" t="inlineStr">
         <is>
+          <t>Energy efficiency</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
           <t>OLADE</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="I34" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1866,40 +1805,37 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K34" s="2">
-        <v>46146</v>
       </c>
     </row>
     <row r="35">
       <c r="A35">
-        <v>1754</v>
+        <v>2023</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Electricity consumption</t>
+          <t>Energy intensity measured in terms of final energy consumption and GDP</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E35" t="inlineStr">
         <is>
+          <t>Energy efficiency</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
           <t>OLADE</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1914,88 +1850,80 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K35" s="2">
-        <v>46146</v>
       </c>
     </row>
     <row r="36">
       <c r="A36">
-        <v>1755</v>
+        <v>4184</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Installed capacity for producing electricity (historical series)</t>
+          <t>Change in energy intensity measured in terms of final energy consumption and GDP</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E36" t="inlineStr">
         <is>
+          <t>Energy efficiency</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
           <t>OLADE</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
           <t>env</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>historical series that ends in 2015 and does not need to be maintained</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37">
-        <v>2023</v>
+        <v>4243</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>GDP energy intensity (Final energy consumption / GDP)</t>
+          <t>Energy intensity measured in terms of final energy consumption and GDP, by economic activity</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>OLADE</t>
+          <t>Energy efficiency</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>ECLAC</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>Energy intensity_Economic activity</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2007,43 +1935,40 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K37" s="2">
-        <v>46136</v>
       </c>
     </row>
     <row r="38">
       <c r="A38">
-        <v>2487</v>
+        <v>4150</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Primary and secondary energy supply</t>
+          <t>Installed electricity-generating capacity, by energy source</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E38" t="inlineStr">
         <is>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
           <t>OLADE</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Type of energy__Primary_and_Secondary</t>
-        </is>
-      </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>Type of energy source</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2060,40 +1985,37 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K38" s="2">
-        <v>46133</v>
       </c>
     </row>
     <row r="39">
       <c r="A39">
-        <v>3154</v>
+        <v>1755</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Renewable proportion of primary energy supply</t>
+          <t>Installed electricity-generating capacity (historical series)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E39" t="inlineStr">
         <is>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
           <t>OLADE</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2104,192 +2026,214 @@
           <t>env</t>
         </is>
       </c>
-      <c r="K39" s="2">
-        <v>46132</v>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>historical series that ends in 2015 and does not need to be maintained</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40">
-        <v>3882</v>
+        <v>1754</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Proportion of population with primary reliance on clean fuels and technology (%) EG_EGY_CLEAN</t>
+          <t>Electricity consumption</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SDG</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>OLADE</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>sdg</t>
+          <t>env</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41">
-        <v>3883</v>
+        <v>4234</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Renewable energy share in the total final energy consumption (%) EG_FEC_RNEW</t>
+          <t>Electricity losses</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SDG</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>OLADE</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>sdg</t>
+          <t>env</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42">
-        <v>4375</v>
+        <v>4235</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Fossil-fuel subsidies (consumption and production) as a proportion of total GDP (%) ER_FFS_CMPT_GDP</t>
+          <t>Electricity losses as a proportion of total electricity supply</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SDG</t>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>OLADE</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>sdg</t>
+          <t>env</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43">
-        <v>4826</v>
+        <v>4244</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Fossil-fuel subsidies (consumption and production) (billions of nominal United States dollars) ER_FFS_CMPT_CD</t>
+          <t>Public investment in renewable energy</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SDG</t>
+          <t>Energy investment and subsidies</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>IRENA</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Type of renewable energy</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>sdg</t>
+          <t>env</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44">
-        <v>4827</v>
+        <v>4826</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Fossil-fuel subsidies (consumption and production) per capita (nominal United States dollars) ER_FFS_CMPT_PC_CD</t>
+          <t>Fossil-fuel subsidies (consumption and production) (billions of nominal United States dollars) ER_FFS_CMPT_CD</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E44" t="inlineStr">
         <is>
+          <t>Energy investment and subsidies</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
           <t>SDG</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>N</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2300,129 +2244,101 @@
     </row>
     <row r="45">
       <c r="A45">
-        <v>5672</v>
+        <v>4375</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Energy production</t>
+          <t>Fossil-fuel subsidies (consumption and production) as a proportion of total GDP (%) ER_FFS_CMPT_GDP</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
           <t>Energy resources</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Production and consumption of energy from non-renewable and renewable sources</t>
-        </is>
-      </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>OLADE</t>
+          <t>Energy investment and subsidies</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Type of energy__Primary_and_Secondary</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>SDG</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="K45" s="2">
-        <v>46135</v>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>this used to be indicator 2040</t>
+          <t>sdg</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46">
-        <v>4252</v>
+        <v>4827</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Share of real Exports of Primary Products according to Renewable and Non-Renewable Natural Resources, and Manufacturing Products in total exports (percentages)</t>
+          <t>Fossil-fuel subsidies (consumption and production) per capita (nominal United States dollars) ER_FFS_CMPT_PC_CD</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Land</t>
+          <t>Environmental resources and their use</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Land use</t>
+          <t>Energy resources</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ECLAC</t>
+          <t>Energy investment and subsidies</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Item - Natural Resources</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>SDG</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>env</t>
+          <t>sdg</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47">
-        <v>4264</v>
+        <v>1739</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Composition of Exports of Primary Products according to Renewable and Non-Renewable Natural Resources, and Manufacturing Products (millions of US $, at constant 2010 prices)</t>
+          <t>Irrigated area</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
           <t>Land</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>Land use</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>ECLAC</t>
-        </is>
-      </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Item - Natural Resources</t>
+          <t>FAO</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -2433,30 +2349,40 @@
     </row>
     <row r="48">
       <c r="A48">
-        <v>4049</v>
+        <v>1869</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Proportion of agricultural area with organic agriculture</t>
+          <t>Agricultural area, by type of land use</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
           <t>Land</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>Land use</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>FAO</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
+          <t>Type of agricultural land</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -2469,43 +2395,35 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K48" s="2">
-        <v>45968</v>
       </c>
     </row>
     <row r="49">
       <c r="A49">
-        <v>1869</v>
+        <v>4049</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Agricultural area</t>
+          <t>Proportion of agricultural area under organic farming</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
           <t>Land</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>Land use</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>FAO</t>
-        </is>
-      </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Type of agricultural land</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>CRED</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2513,44 +2431,51 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="J49" t="inlineStr">
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K49" s="2">
-        <v>45960</v>
       </c>
     </row>
     <row r="50">
       <c r="A50">
-        <v>1739</v>
+        <v>2019</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Irrigated area</t>
+          <t>Capture fisheries production</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Land</t>
+          <t>Environmental resources and their use</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Land use</t>
+          <t>Biological resources</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
+          <t>Aquatic resources</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
           <t>FAO</t>
         </is>
       </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Type of fishery</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I50" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2560,43 +2485,40 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K50" s="2">
-        <v>45999</v>
       </c>
     </row>
     <row r="51">
       <c r="A51">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Fish capture production</t>
+          <t>Aquaculture production</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
           <t>Biological resources</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Aquatic resources and their use</t>
-        </is>
-      </c>
       <c r="E51" t="inlineStr">
         <is>
+          <t>Aquatic resources</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
           <t>FAO</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Type of fishery</t>
-        </is>
-      </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>Aquaculture production area</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2613,43 +2535,40 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K51" s="2">
-        <v>45982</v>
       </c>
     </row>
     <row r="52">
       <c r="A52">
-        <v>2020</v>
+        <v>1740</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Aquaculture production</t>
+          <t>Harvested area of main crops</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
           <t>Biological resources</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Aquatic resources and their use</t>
-        </is>
-      </c>
       <c r="E52" t="inlineStr">
         <is>
+          <t>Crops</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
           <t>FAO</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>Aquaculture production area</t>
-        </is>
-      </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>Crop</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2666,84 +2585,73 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K52" s="2">
-        <v>45982</v>
       </c>
     </row>
     <row r="53">
       <c r="A53">
-        <v>2022</v>
+        <v>2038</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Fertilizer use intensity</t>
+          <t>Fertilizer consumption</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
           <t>Biological resources</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>Crops</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>FAO</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="J53" t="inlineStr">
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K53" s="2">
-        <v>45968</v>
       </c>
     </row>
     <row r="54">
       <c r="A54">
-        <v>3382</v>
+        <v>2022</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Pesticide use intensity</t>
+          <t>Fertilizer use intensity</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
           <t>Biological resources</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>Crops</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>FAO</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>ECLAC</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2757,48 +2665,40 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K54" s="2">
-        <v>45968</v>
       </c>
     </row>
     <row r="55">
       <c r="A55">
-        <v>1740</v>
+        <v>2039</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Harvested area of main crops</t>
+          <t>Pesticide consumption</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
           <t>Biological resources</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="E55" t="inlineStr">
         <is>
           <t>Crops</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>FAO</t>
-        </is>
-      </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Crop</t>
+          <t>ECLAC</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>Type of Pesticide</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -2810,36 +2710,38 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K55" s="2">
-        <v>45960</v>
       </c>
     </row>
     <row r="56">
       <c r="A56">
-        <v>2038</v>
+        <v>3382</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Fertilizer consumption</t>
+          <t>Pesticide use intensity</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
           <t>Biological resources</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>Crops</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>FAO</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>ECLAC</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2848,57 +2750,46 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K56" s="2">
-        <v>45999</v>
       </c>
     </row>
     <row r="57">
       <c r="A57">
-        <v>2039</v>
+        <v>3853</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Pesticide consumption</t>
+          <t>Level of water stress: freshwater withdrawal as a proportion of available freshwater resources (%) ER_H2O_STRESS</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Biological resources</t>
+          <t>Environmental resources and their use</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Crops</t>
+          <t>Water resources</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>FAO</t>
+          <t>Water resources</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Type of Pesticide</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>SDG</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Activity</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="K57" s="2">
-        <v>46113</v>
+          <t>sdg</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -2907,35 +2798,35 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Sectoral distribution of water extraction</t>
+          <t>Water withdrawal, by sector</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
           <t>Water resources</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>Abstraction, use and returns of water</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>FAO</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="G58" t="inlineStr">
         <is>
           <t>Sector__Water resources</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
+      <c r="H58" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2944,9 +2835,6 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K58" s="2">
-        <v>45985</v>
       </c>
     </row>
     <row r="59">
@@ -2955,30 +2843,30 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Water intensity of agricultural added value</t>
+          <t>Water intensity of agricultural value added</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
           <t>Water resources</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>Abstraction, use and returns of water</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>FAO</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>ECLAC</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2987,9 +2875,6 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K59" s="2">
-        <v>45985</v>
       </c>
     </row>
     <row r="60">
@@ -3003,32 +2888,32 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
           <t>Water resources</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="E60" t="inlineStr">
         <is>
           <t>Abstraction, use and returns of water</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="F60" t="inlineStr">
         <is>
           <t>SDG</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="G60" t="inlineStr">
         <is>
           <t>Activity</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>N</t>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -3039,31 +2924,36 @@
     </row>
     <row r="61">
       <c r="A61">
-        <v>3850</v>
+        <v>3855</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Proportion of bodies of water with good ambient water quality (%) EN_H2O_WBAMBQ</t>
+          <t>Degree of integrated water resources management implementation (%) ER_H2O_IWRMD</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
+          <t>Environmental resources and their use</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
           <t>Water resources</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>Abstraction, use and returns of water</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
+      <c r="F61" t="inlineStr">
         <is>
           <t>SDG</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>N</t>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Level/Status</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3074,116 +2964,126 @@
     </row>
     <row r="62">
       <c r="A62">
-        <v>3853</v>
+        <v>3387</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Level of water stress: freshwater withdrawal as a proportion of available freshwater resources (%) ER_H2O_STRESS</t>
+          <t>Share of global greenhouse gas (GHG) emissions</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Water resources</t>
+          <t>Residuals</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Abstraction, use and returns of water</t>
+          <t>Emissions to air</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>SDG</t>
+          <t>Emissions of greenhouse gases (GHGs)</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>N</t>
+          <t>CAIT - WRI</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>sdg</t>
+          <t>env</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63">
-        <v>3855</v>
+        <v>3351</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Degree of integrated water resources management implementation (%) ER_H2O_IWRMD</t>
+          <t>Greenhouse gas (GHG) emissions, by sector</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Water resources</t>
+          <t>Residuals</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Abstraction, use and returns of water</t>
+          <t>Emissions to air</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>SDG</t>
+          <t>Emissions of greenhouse gases (GHGs)</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Level/Status</t>
+          <t>CAIT - WRI</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Greenhouse Gas (GHG) Emissions by sector</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>sdg</t>
+          <t>env</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64">
-        <v>4501</v>
+        <v>4462</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Lakes and rivers permanent water area (square kilometres) EN_LKRV_PWAN</t>
+          <t>Greenhouse gas (GHG) emissions from the energy sector</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Water resources</t>
+          <t>Residuals</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Abstraction, use and returns of water</t>
+          <t>Emissions to air</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>SDG</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>N</t>
+          <t>Emissions of greenhouse gases (GHGs)</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>CAIT - WRI</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Greenhouse Gas (GHG) Emissions of the energy sector</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>sdg</t>
+          <t>env</t>
         </is>
       </c>
     </row>
@@ -3193,72 +3093,64 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Greenhouse Gas (GHG) emissions of GDP</t>
+          <t>Greenhouse gas (GHG) emissions per unit of GDP</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Waste</t>
+          <t>Residuals</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Air emissions / Emissions of greenhouse gases (GHGs)</t>
+          <t>Emissions to air</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
+          <t>Emissions of greenhouse gases (GHGs)</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
           <t>CAIT - WRI</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>Greenhouse Gas (GHG) Emissions of GDP</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="J65" t="inlineStr">
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K65" s="2">
-        <v>46020</v>
       </c>
     </row>
     <row r="66">
       <c r="A66">
-        <v>4462</v>
+        <v>4461</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Greenhouse Gas (GHG) emissions of the energy sector</t>
+          <t>Greenhouse gas (GHG) emissions per capita</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Waste</t>
+          <t>Residuals</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Air emissions / Emissions of greenhouse gases (GHGs)</t>
+          <t>Emissions to air</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
+          <t>Emissions of greenhouse gases (GHGs)</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
           <t>CAIT - WRI</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>Greenhouse Gas (GHG) Emissions of the energy sector</t>
-        </is>
-      </c>
       <c r="I66" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3268,32 +3160,34 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K66" s="2">
-        <v>46029</v>
       </c>
     </row>
     <row r="67">
       <c r="A67">
-        <v>4461</v>
+        <v>3158</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Greenhouse gas (GHG) emissions per capita</t>
+          <t>Carbon dioxide (CO2) emissions, excluding land-use change and forestry</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Waste</t>
+          <t>Residuals</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Air emissions / Emissions of greenhouse gases (GHGs)</t>
+          <t>Emissions to air</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
+          <t>Emissions of greenhouse gases (GHGs)</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
           <t>CAIT - WRI</t>
         </is>
       </c>
@@ -3302,45 +3196,42 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="J67" t="inlineStr">
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K67" s="2">
-        <v>46001</v>
       </c>
     </row>
     <row r="68">
       <c r="A68">
-        <v>5649</v>
+        <v>3159</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Carbon dioxide (CO2) emissions per capita</t>
+          <t>Share of global carbon dioxide (CO2) emissions</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Waste</t>
+          <t>Residuals</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Air emissions / Emissions of greenhouse gases (GHGs)</t>
+          <t>Emissions to air</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
+          <t>Emissions of greenhouse gases (GHGs)</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
           <t>CAIT - WRI</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr">
+      <c r="H68" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3349,9 +3240,6 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K68" s="2">
-        <v>45980</v>
       </c>
     </row>
     <row r="69">
@@ -3360,25 +3248,30 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Carbon dioxide (CO2) emissions per GDP</t>
+          <t>Carbon dioxide (CO2) emissions per unit of GDP</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Waste</t>
+          <t>Residuals</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Air emissions / Emissions of greenhouse gases (GHGs)</t>
+          <t>Emissions to air</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
+          <t>Emissions of greenhouse gases (GHGs)</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
           <t>CAIT - WRI</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr">
+      <c r="H69" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3387,41 +3280,38 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K69" s="2">
-        <v>45980</v>
       </c>
     </row>
     <row r="70">
       <c r="A70">
-        <v>3158</v>
+        <v>5649</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Carbon dioxide (CO2) emissions, total excluding land change use and forestry</t>
+          <t>Carbon dioxide (CO2) emissions per capita</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Waste</t>
+          <t>Residuals</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Air emissions / Emissions of greenhouse gases (GHGs)</t>
+          <t>Emissions to air</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
+          <t>Emissions of greenhouse gases (GHGs)</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
           <t>CAIT - WRI</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>Carbon dioxide (CO2) emissions</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
+      <c r="H70" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3430,37 +3320,44 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K70" s="2">
-        <v>45980</v>
       </c>
     </row>
     <row r="71">
       <c r="A71">
-        <v>3159</v>
+        <v>2037</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Proportion of carbon dioxide (CO2) emissions in relation to global emissions</t>
+          <t>Consumption of all ozone-depleting substances (ODS)</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Waste</t>
+          <t>Residuals</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Air emissions / Emissions of greenhouse gases (GHGs)</t>
+          <t>Emissions to air</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>CAIT - WRI</t>
+          <t>Consumption of ozone depleting substances (ODS)</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>UNEP</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
+          <t>Type of ozone depleting substances (ODS)</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
@@ -3473,43 +3370,35 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K71" s="2">
-        <v>45974</v>
       </c>
     </row>
     <row r="72">
       <c r="A72">
-        <v>3351</v>
+        <v>3852</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Greenhouse gas (GHG) emissions by sector</t>
+          <t>Proportion of safely treated domestic wastewater flows (%) EN_WWT_WWDS</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Waste</t>
+          <t>Residuals</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Air emissions / Emissions of greenhouse gases (GHGs)</t>
+          <t>Generation and management of wastewater</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>CAIT - WRI</t>
+          <t>Collection and treatment of wastewater</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Greenhouse Gas (GHG) Emissions by sector</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>SDG</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -3517,218 +3406,214 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="K72" s="2">
-        <v>45981</v>
+          <t>sdg</t>
+        </is>
       </c>
     </row>
     <row r="73">
       <c r="A73">
-        <v>3387</v>
+        <v>4370</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Proportion of geenhouse gas emissions (GHG) in relation to global emissions</t>
+          <t>Municipal waste recycled (Tonnes) EN_MWT_RCYV</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Waste</t>
+          <t>Residuals</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Air emissions / Emissions of greenhouse gases (GHGs)</t>
+          <t>Generation and management of waste</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>CAIT - WRI</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>Management of waste</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>SDG</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="K73" s="2">
-        <v>46003</v>
+          <t>sdg</t>
+        </is>
       </c>
     </row>
     <row r="74">
       <c r="A74">
-        <v>2037</v>
+        <v>5113</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Consumption of ozone depleting substances (ODS)</t>
+          <t>Electronic waste recycled (Tonnes) EN_EWT_RCYV</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Waste</t>
+          <t>Residuals</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Air emissions</t>
+          <t>Generation and management of waste</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>UNEP</t>
+          <t>Management of waste</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Type of ozone depleting substances (ODS)</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>SDG</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="K74" s="2">
-        <v>46044</v>
+          <t>sdg</t>
+        </is>
       </c>
     </row>
     <row r="75">
       <c r="A75">
-        <v>3852</v>
+        <v>5647</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Proportion of safely treated domestic wastewater flows (%) EN_WWT_WWDS</t>
+          <t>Number of disaster events, by type of disaster</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Waste</t>
+          <t>Extreme events and disasters</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Sewage water</t>
+          <t>Natural extreme events and disasters</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>SDG</t>
+          <t>Occurrence of natural extreme events and disasters</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>CRED</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>N</t>
+          <t>Type of disaster</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>sdg</t>
+          <t>env</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76">
-        <v>4370</v>
+        <v>5645</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Municipal waste recycled (Tonnes) EN_MWT_RCYV</t>
+          <t>Number of deaths attributed to disasters, by type of disaster</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Waste</t>
+          <t>Extreme events and disasters</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Waste</t>
+          <t>Natural extreme events and disasters</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>SDG</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>N</t>
+          <t>Impact of natural extreme events and disasters</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>CRED</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Type of disaster</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>sdg</t>
+          <t>env</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77">
-        <v>5113</v>
+        <v>5646</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Electronic waste recycled (Tonnes) EN_EWT_RCYV</t>
+          <t>Number of directly affected persons attributed to disasters, by type of disaster</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Waste</t>
+          <t>Extreme events and disasters</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Waste</t>
+          <t>Natural extreme events and disasters</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>SDG</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>N</t>
+          <t>Impact of natural extreme events and disasters</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>CRED</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Type of disaster</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>sdg</t>
+          <t>env</t>
         </is>
       </c>
     </row>
@@ -3738,35 +3623,35 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Economic cost of disasters, by type of disaster_x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D__x000D_
+          <t xml:space="preserve">Economic loss attributed to disasters, by type of disaster
 </t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
+          <t>Extreme events and disasters</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
           <t>Natural extreme events and disasters</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Occurrence and impact of disasters</t>
-        </is>
-      </c>
       <c r="E78" t="inlineStr">
         <is>
+          <t>Impact of natural extreme events and disasters</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
           <t>CRED</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr">
+      <c r="G78" t="inlineStr">
         <is>
           <t>Type of disaster</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="H78" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3781,81 +3666,75 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K78" s="2">
-        <v>45986</v>
       </c>
     </row>
     <row r="79">
       <c r="A79">
-        <v>5647</v>
+        <v>3882</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Number of disaster events, by type of disaster</t>
+          <t>Proportion of population with primary reliance on clean fuels and technology (%) EG_EGY_CLEAN</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Natural extreme events and disasters</t>
+          <t>Human settlements and environmental health</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Occurrence and impact of disasters</t>
+          <t>Human settlements</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>CRED</t>
+          <t>Access to selected basic services</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Type of disaster</t>
-        </is>
-      </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>SDG</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Location</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="K79" s="2">
-        <v>45968</v>
+          <t>sdg</t>
+        </is>
       </c>
     </row>
     <row r="80">
       <c r="A80">
-        <v>5645</v>
+        <v>1763</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Human deaths caused by disasters, by type of disaster</t>
+          <t>ISO 14001-certified enterprises</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Natural extreme events and disasters</t>
+          <t>Environmental protection, management and engagement</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Occurrence and impact of disasters</t>
+          <t>Environmental governance and regulation</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>CRED</t>
+          <t>Environmental regulation and instruments</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Type of disaster</t>
+          <t>ISO</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -3867,86 +3746,90 @@
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K80" s="2">
-        <v>45968</v>
       </c>
     </row>
     <row r="81">
       <c r="A81">
-        <v>5646</v>
+        <v>2029</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Persons directly affected by disasters, by type of disaster</t>
+          <t>ISO 14001-certified enterprises per unit of GDP</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Natural extreme events and disasters</t>
+          <t>Environmental protection, management and engagement</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Occurrence and impact of disasters</t>
+          <t>Environmental governance and regulation</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>CRED</t>
+          <t>Environmental regulation and instruments</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Type of disaster</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>ECLAC</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
           <t>env</t>
         </is>
-      </c>
-      <c r="K81" s="2">
-        <v>45968</v>
       </c>
     </row>
     <row r="82">
       <c r="A82">
-        <v>3724</v>
+        <v>2031</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Score of adoption and implementation of national DRR strategies in line with the Sendai Framework SG_DSR_LGRGSR</t>
+          <t>Multilateral environmental agreements</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Natural extreme events and disasters</t>
+          <t>Environmental protection, management and engagement</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Occurrence and impact of disasters</t>
+          <t>Environmental governance and regulation</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>SDG</t>
+          <t>Participation in MEAs and environmental conventions</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>InforMEA</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Multilateral environmental agreements; Signature, party, entry into force</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>sdg</t>
+          <t>env</t>
         </is>
       </c>
     </row>
@@ -3961,22 +3844,22 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Natural extreme events and disasters</t>
+          <t>Environmental protection, management and engagement</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Occurrence and impact of disasters</t>
+          <t>Extreme event preparedness and disaster management</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
+          <t>Preparedness for natural extreme events and disasters</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
           <t>SDG</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>N</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -3987,414 +3870,46 @@
     </row>
     <row r="84">
       <c r="A84">
-        <v>1763</v>
+        <v>3724</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>ISO 14001-certified enterprises</t>
+          <t>Score of adoption and implementation of national DRR strategies in line with the Sendai Framework SG_DSR_LGRGSR</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Environmental governance and regulation</t>
+          <t>Environmental protection, management and engagement</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Environmental regulation and instruments</t>
+          <t>Extreme event preparedness and disaster management</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>ISO</t>
-        </is>
-      </c>
-      <c r="H84" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>Preparedness for natural extreme events and disasters</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>SDG</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="K84" s="2">
-        <v>46044</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85">
-        <v>2029</v>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>ISO 14001-certified enterprises per billion dollars of GDP</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>Environmental governance and regulation</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Environmental regulation and instruments</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>ECLAC</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="K85" s="2">
-        <v>46044</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86">
-        <v>2031</v>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>Multilateral environmental agreements</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>Environmental governance and regulation</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>Participation in MEAs and environmental conventions</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>ECLAC</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>Multilateral environmental agreements; Signature, party, entry into force</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="K86" s="2">
-        <v>46092</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87">
-        <v>5731</v>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>Proportion of Marine Key Biodiviersity Areas (KBAs) covered by protected areas</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>ECLAC</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J87" t="inlineStr">
-        <is>
-          <t>coral</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88">
-        <v>5732</v>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>Proportion of coral ecosystems covered by protected areas</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>ECLAC</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>coral</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89">
-        <v>5733</v>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>Monthly mean Sea Surface Temperature (SST) Anomaly</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>ECLAC</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J89" t="inlineStr">
-        <is>
-          <t>coral</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90">
-        <v>5734</v>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>Maximum monthly Sea Surface Temperature (SST) Anomaly</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>ECLAC</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t>coral</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91">
-        <v>5735</v>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>Maximum monthly Coral Bleaching HotSpot</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>ECLAC</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J91" t="inlineStr">
-        <is>
-          <t>coral</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92">
-        <v>5736</v>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>Maximum monthly Degree Heating Week (DHW)</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>ECLAC</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J92" t="inlineStr">
-        <is>
-          <t>coral</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93">
-        <v>5737</v>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>Monthly mean Sea Surface Temperature (SST) Anomaly, by coral ecosystem</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>ECLAC</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J93" t="inlineStr">
-        <is>
-          <t>coral</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94">
-        <v>5738</v>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>Maximum monthly Sea Surface Temperature (SST) Anomaly, by coral ecosystem</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>ECLAC</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J94" t="inlineStr">
-        <is>
-          <t>coral</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95">
-        <v>5739</v>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>Maximum monthly Coral Bleaching HotSpot, by coral ecosystem</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>ECLAC</t>
-        </is>
-      </c>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J95" t="inlineStr">
-        <is>
-          <t>coral</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96">
-        <v>5740</v>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>Maximum monthly Degree Heating Week (DHW), by coral ecosystem</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>ECLAC</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="J96" t="inlineStr">
-        <is>
-          <t>coral</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97">
-        <v>4299</v>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>Total greenhouse gas emissions without LULUCF for non-Annex I Parties (Mt CO2 equivalent) EN_ATM_GHGT_NAIP</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>Waste</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>Air emissions / Emissions of greenhouse gases (GHGs)</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>SDG</t>
+          <t>sdg</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{8b77875e-5908-45a0-9cb4-dec9ae074618}" enabled="1" method="Privileged" siteId="{0f9e35db-544f-4f60-bdcc-5ea416e6dc70}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>